<commit_message>
chore: rebrand Process Schedule to Process Insight
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/process_schedule.xlsx
+++ b/process_schedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Desktop\Apps\Dev\Process_Schedule\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD0DE4D3-B3BE-4267-9149-8E65A9F85B5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0EA8C40-32ED-42CB-9BEB-EAD62B16B1A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6780" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{7AFCA38D-DA68-4C4C-A0AE-17A7CD592C6C}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="22695" windowHeight="14476" xr2:uid="{7AFCA38D-DA68-4C4C-A0AE-17A7CD592C6C}"/>
   </bookViews>
   <sheets>
     <sheet name="Rev.1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="90">
   <si>
     <t>No</t>
     <phoneticPr fontId="1"/>
@@ -591,20 +591,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>実績２</t>
-    <rPh sb="0" eb="2">
-      <t>ジッセキ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>実績３</t>
-    <rPh sb="0" eb="2">
-      <t>ジッセキ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>工程管理パート</t>
     <rPh sb="0" eb="2">
       <t>コウテイ</t>
@@ -629,6 +615,30 @@
     <rPh sb="0" eb="4">
       <t>キホンジョウホウ</t>
     </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>調達BOM入手する</t>
+    <rPh sb="0" eb="2">
+      <t>チョウタツ</t>
+    </rPh>
+    <rPh sb="5" eb="7">
+      <t>ニュウシュ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>開発BOMがどうなっているか確認する</t>
+    <rPh sb="0" eb="2">
+      <t>カイハツ</t>
+    </rPh>
+    <rPh sb="14" eb="16">
+      <t>カクニン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>V2とか</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -819,12 +829,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="55" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -841,6 +845,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="55" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1192,256 +1202,256 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:79" x14ac:dyDescent="0.7">
-      <c r="B3" s="15" t="s">
-        <v>88</v>
-      </c>
-      <c r="C3" s="16"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="16"/>
-      <c r="F3" s="16"/>
-      <c r="G3" s="16"/>
-      <c r="H3" s="17"/>
-      <c r="I3" s="13" t="s">
+      <c r="B3" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="J3" s="13"/>
-      <c r="K3" s="13"/>
-      <c r="L3" s="13"/>
-      <c r="M3" s="13"/>
-      <c r="N3" s="13"/>
-      <c r="O3" s="13"/>
-      <c r="P3" s="13"/>
-      <c r="Q3" s="13"/>
-      <c r="R3" s="13"/>
-      <c r="S3" s="13"/>
-      <c r="T3" s="13"/>
-      <c r="U3" s="13"/>
-      <c r="V3" s="13"/>
-      <c r="W3" s="13"/>
-      <c r="X3" s="13"/>
-      <c r="Y3" s="13"/>
-      <c r="Z3" s="13"/>
-      <c r="AA3" s="13"/>
-      <c r="AB3" s="13"/>
-      <c r="AC3" s="13"/>
-      <c r="AD3" s="13"/>
-      <c r="AE3" s="13"/>
-      <c r="AF3" s="13"/>
-      <c r="AG3" s="13"/>
-      <c r="AH3" s="13"/>
-      <c r="AI3" s="13"/>
-      <c r="AJ3" s="13"/>
-      <c r="AK3" s="13"/>
-      <c r="AL3" s="13" t="s">
-        <v>87</v>
-      </c>
-      <c r="AM3" s="13"/>
-      <c r="AN3" s="13"/>
-      <c r="AO3" s="13"/>
-      <c r="AP3" s="13"/>
-      <c r="AQ3" s="13"/>
-      <c r="AR3" s="13"/>
-      <c r="AS3" s="13"/>
-      <c r="AT3" s="13"/>
-      <c r="AU3" s="13"/>
-      <c r="AV3" s="13"/>
-      <c r="AW3" s="13"/>
-      <c r="AX3" s="14">
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+      <c r="H3" s="15"/>
+      <c r="I3" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="J3" s="19"/>
+      <c r="K3" s="19"/>
+      <c r="L3" s="19"/>
+      <c r="M3" s="19"/>
+      <c r="N3" s="19"/>
+      <c r="O3" s="19"/>
+      <c r="P3" s="19"/>
+      <c r="Q3" s="19"/>
+      <c r="R3" s="19"/>
+      <c r="S3" s="19"/>
+      <c r="T3" s="19"/>
+      <c r="U3" s="19"/>
+      <c r="V3" s="19"/>
+      <c r="W3" s="19"/>
+      <c r="X3" s="19"/>
+      <c r="Y3" s="19"/>
+      <c r="Z3" s="19"/>
+      <c r="AA3" s="19"/>
+      <c r="AB3" s="19"/>
+      <c r="AC3" s="19"/>
+      <c r="AD3" s="19"/>
+      <c r="AE3" s="19"/>
+      <c r="AF3" s="19"/>
+      <c r="AG3" s="19"/>
+      <c r="AH3" s="19"/>
+      <c r="AI3" s="19"/>
+      <c r="AJ3" s="19"/>
+      <c r="AK3" s="19"/>
+      <c r="AL3" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="AM3" s="19"/>
+      <c r="AN3" s="19"/>
+      <c r="AO3" s="19"/>
+      <c r="AP3" s="19"/>
+      <c r="AQ3" s="19"/>
+      <c r="AR3" s="19"/>
+      <c r="AS3" s="19"/>
+      <c r="AT3" s="19"/>
+      <c r="AU3" s="19"/>
+      <c r="AV3" s="19"/>
+      <c r="AW3" s="19"/>
+      <c r="AX3" s="20">
         <v>45748</v>
       </c>
-      <c r="AY3" s="14"/>
-      <c r="AZ3" s="14"/>
-      <c r="BA3" s="14"/>
-      <c r="BB3" s="14"/>
-      <c r="BC3" s="14"/>
-      <c r="BD3" s="14"/>
-      <c r="BE3" s="14"/>
-      <c r="BF3" s="14"/>
-      <c r="BG3" s="14"/>
-      <c r="BH3" s="14"/>
-      <c r="BI3" s="14"/>
-      <c r="BJ3" s="14"/>
-      <c r="BK3" s="14"/>
-      <c r="BL3" s="14"/>
-      <c r="BM3" s="14"/>
-      <c r="BN3" s="14"/>
-      <c r="BO3" s="14"/>
-      <c r="BP3" s="14"/>
-      <c r="BQ3" s="14"/>
-      <c r="BR3" s="14"/>
-      <c r="BS3" s="14"/>
-      <c r="BT3" s="14"/>
-      <c r="BU3" s="14"/>
-      <c r="BV3" s="14"/>
-      <c r="BW3" s="14"/>
-      <c r="BX3" s="14"/>
-      <c r="BY3" s="14"/>
-      <c r="BZ3" s="14"/>
-      <c r="CA3" s="14"/>
+      <c r="AY3" s="20"/>
+      <c r="AZ3" s="20"/>
+      <c r="BA3" s="20"/>
+      <c r="BB3" s="20"/>
+      <c r="BC3" s="20"/>
+      <c r="BD3" s="20"/>
+      <c r="BE3" s="20"/>
+      <c r="BF3" s="20"/>
+      <c r="BG3" s="20"/>
+      <c r="BH3" s="20"/>
+      <c r="BI3" s="20"/>
+      <c r="BJ3" s="20"/>
+      <c r="BK3" s="20"/>
+      <c r="BL3" s="20"/>
+      <c r="BM3" s="20"/>
+      <c r="BN3" s="20"/>
+      <c r="BO3" s="20"/>
+      <c r="BP3" s="20"/>
+      <c r="BQ3" s="20"/>
+      <c r="BR3" s="20"/>
+      <c r="BS3" s="20"/>
+      <c r="BT3" s="20"/>
+      <c r="BU3" s="20"/>
+      <c r="BV3" s="20"/>
+      <c r="BW3" s="20"/>
+      <c r="BX3" s="20"/>
+      <c r="BY3" s="20"/>
+      <c r="BZ3" s="20"/>
+      <c r="CA3" s="20"/>
     </row>
     <row r="4" spans="2:79" x14ac:dyDescent="0.7">
-      <c r="B4" s="18"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
-      <c r="G4" s="19"/>
-      <c r="H4" s="20"/>
-      <c r="I4" s="13"/>
-      <c r="J4" s="13"/>
-      <c r="K4" s="13"/>
-      <c r="L4" s="13"/>
-      <c r="M4" s="13"/>
-      <c r="N4" s="13"/>
-      <c r="O4" s="13"/>
-      <c r="P4" s="13"/>
-      <c r="Q4" s="13"/>
-      <c r="R4" s="13"/>
-      <c r="S4" s="13"/>
-      <c r="T4" s="13"/>
-      <c r="U4" s="13"/>
-      <c r="V4" s="13"/>
-      <c r="W4" s="13"/>
-      <c r="X4" s="13"/>
-      <c r="Y4" s="13"/>
-      <c r="Z4" s="13"/>
-      <c r="AA4" s="13"/>
-      <c r="AB4" s="13"/>
-      <c r="AC4" s="13"/>
-      <c r="AD4" s="13"/>
-      <c r="AE4" s="13"/>
-      <c r="AF4" s="13"/>
-      <c r="AG4" s="13"/>
-      <c r="AH4" s="13"/>
-      <c r="AI4" s="13"/>
-      <c r="AJ4" s="13"/>
-      <c r="AK4" s="13"/>
-      <c r="AL4" s="13"/>
-      <c r="AM4" s="13"/>
-      <c r="AN4" s="13"/>
-      <c r="AO4" s="13"/>
-      <c r="AP4" s="13"/>
-      <c r="AQ4" s="13"/>
-      <c r="AR4" s="13"/>
-      <c r="AS4" s="13"/>
-      <c r="AT4" s="13"/>
-      <c r="AU4" s="13"/>
-      <c r="AV4" s="13"/>
-      <c r="AW4" s="13"/>
-      <c r="AX4" s="13"/>
-      <c r="AY4" s="13"/>
-      <c r="AZ4" s="13"/>
-      <c r="BA4" s="13"/>
-      <c r="BB4" s="13"/>
-      <c r="BC4" s="13"/>
-      <c r="BD4" s="13"/>
-      <c r="BE4" s="13"/>
-      <c r="BF4" s="13"/>
-      <c r="BG4" s="13"/>
-      <c r="BH4" s="13"/>
-      <c r="BI4" s="13"/>
-      <c r="BJ4" s="13"/>
-      <c r="BK4" s="13"/>
-      <c r="BL4" s="13"/>
-      <c r="BM4" s="13"/>
-      <c r="BN4" s="13"/>
-      <c r="BO4" s="13"/>
-      <c r="BP4" s="13"/>
-      <c r="BQ4" s="13"/>
-      <c r="BR4" s="13"/>
-      <c r="BS4" s="13"/>
-      <c r="BT4" s="13"/>
-      <c r="BU4" s="13"/>
-      <c r="BV4" s="13"/>
-      <c r="BW4" s="13"/>
-      <c r="BX4" s="13"/>
-      <c r="BY4" s="13"/>
-      <c r="BZ4" s="13"/>
-      <c r="CA4" s="13"/>
+      <c r="B4" s="16"/>
+      <c r="C4" s="17"/>
+      <c r="D4" s="17"/>
+      <c r="E4" s="17"/>
+      <c r="F4" s="17"/>
+      <c r="G4" s="17"/>
+      <c r="H4" s="18"/>
+      <c r="I4" s="19"/>
+      <c r="J4" s="19"/>
+      <c r="K4" s="19"/>
+      <c r="L4" s="19"/>
+      <c r="M4" s="19"/>
+      <c r="N4" s="19"/>
+      <c r="O4" s="19"/>
+      <c r="P4" s="19"/>
+      <c r="Q4" s="19"/>
+      <c r="R4" s="19"/>
+      <c r="S4" s="19"/>
+      <c r="T4" s="19"/>
+      <c r="U4" s="19"/>
+      <c r="V4" s="19"/>
+      <c r="W4" s="19"/>
+      <c r="X4" s="19"/>
+      <c r="Y4" s="19"/>
+      <c r="Z4" s="19"/>
+      <c r="AA4" s="19"/>
+      <c r="AB4" s="19"/>
+      <c r="AC4" s="19"/>
+      <c r="AD4" s="19"/>
+      <c r="AE4" s="19"/>
+      <c r="AF4" s="19"/>
+      <c r="AG4" s="19"/>
+      <c r="AH4" s="19"/>
+      <c r="AI4" s="19"/>
+      <c r="AJ4" s="19"/>
+      <c r="AK4" s="19"/>
+      <c r="AL4" s="19"/>
+      <c r="AM4" s="19"/>
+      <c r="AN4" s="19"/>
+      <c r="AO4" s="19"/>
+      <c r="AP4" s="19"/>
+      <c r="AQ4" s="19"/>
+      <c r="AR4" s="19"/>
+      <c r="AS4" s="19"/>
+      <c r="AT4" s="19"/>
+      <c r="AU4" s="19"/>
+      <c r="AV4" s="19"/>
+      <c r="AW4" s="19"/>
+      <c r="AX4" s="19"/>
+      <c r="AY4" s="19"/>
+      <c r="AZ4" s="19"/>
+      <c r="BA4" s="19"/>
+      <c r="BB4" s="19"/>
+      <c r="BC4" s="19"/>
+      <c r="BD4" s="19"/>
+      <c r="BE4" s="19"/>
+      <c r="BF4" s="19"/>
+      <c r="BG4" s="19"/>
+      <c r="BH4" s="19"/>
+      <c r="BI4" s="19"/>
+      <c r="BJ4" s="19"/>
+      <c r="BK4" s="19"/>
+      <c r="BL4" s="19"/>
+      <c r="BM4" s="19"/>
+      <c r="BN4" s="19"/>
+      <c r="BO4" s="19"/>
+      <c r="BP4" s="19"/>
+      <c r="BQ4" s="19"/>
+      <c r="BR4" s="19"/>
+      <c r="BS4" s="19"/>
+      <c r="BT4" s="19"/>
+      <c r="BU4" s="19"/>
+      <c r="BV4" s="19"/>
+      <c r="BW4" s="19"/>
+      <c r="BX4" s="19"/>
+      <c r="BY4" s="19"/>
+      <c r="BZ4" s="19"/>
+      <c r="CA4" s="19"/>
     </row>
     <row r="5" spans="2:79" x14ac:dyDescent="0.7">
-      <c r="B5" s="13" t="s">
+      <c r="B5" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="C5" s="13"/>
-      <c r="D5" s="13" t="s">
+      <c r="C5" s="19"/>
+      <c r="D5" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="E5" s="13" t="s">
+      <c r="E5" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="F5" s="13" t="s">
+      <c r="F5" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="G5" s="13" t="s">
+      <c r="G5" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="H5" s="13" t="s">
+      <c r="H5" s="19" t="s">
         <v>5</v>
       </c>
       <c r="I5" s="2"/>
       <c r="J5" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="K5" s="13" t="s">
+      <c r="K5" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="L5" s="13"/>
-      <c r="M5" s="13"/>
-      <c r="N5" s="13"/>
-      <c r="O5" s="13"/>
-      <c r="P5" s="13" t="s">
+      <c r="L5" s="19"/>
+      <c r="M5" s="19"/>
+      <c r="N5" s="19"/>
+      <c r="O5" s="19"/>
+      <c r="P5" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="Q5" s="13"/>
-      <c r="R5" s="13"/>
-      <c r="S5" s="13"/>
-      <c r="T5" s="13"/>
-      <c r="U5" s="13"/>
-      <c r="V5" s="13"/>
-      <c r="W5" s="13"/>
-      <c r="X5" s="13"/>
-      <c r="Y5" s="13"/>
+      <c r="Q5" s="19"/>
+      <c r="R5" s="19"/>
+      <c r="S5" s="19"/>
+      <c r="T5" s="19"/>
+      <c r="U5" s="19"/>
+      <c r="V5" s="19"/>
+      <c r="W5" s="19"/>
+      <c r="X5" s="19"/>
+      <c r="Y5" s="19"/>
       <c r="Z5" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="AA5" s="13" t="s">
+      <c r="AA5" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="AB5" s="13"/>
-      <c r="AC5" s="13" t="s">
+      <c r="AB5" s="19"/>
+      <c r="AC5" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="AD5" s="13"/>
-      <c r="AE5" s="13" t="s">
+      <c r="AD5" s="19"/>
+      <c r="AE5" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="AF5" s="13"/>
-      <c r="AG5" s="13"/>
+      <c r="AF5" s="19"/>
+      <c r="AG5" s="19"/>
       <c r="AH5" s="2" t="s">
         <v>35</v>
       </c>
       <c r="AI5" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="AJ5" s="13" t="s">
+      <c r="AJ5" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="AK5" s="13" t="s">
+      <c r="AK5" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="AL5" s="13"/>
-      <c r="AM5" s="13"/>
-      <c r="AN5" s="13"/>
-      <c r="AO5" s="13"/>
-      <c r="AP5" s="13"/>
-      <c r="AQ5" s="13"/>
-      <c r="AR5" s="13"/>
-      <c r="AS5" s="13"/>
-      <c r="AT5" s="13"/>
-      <c r="AU5" s="13"/>
-      <c r="AV5" s="13"/>
-      <c r="AW5" s="13"/>
+      <c r="AL5" s="19"/>
+      <c r="AM5" s="19"/>
+      <c r="AN5" s="19"/>
+      <c r="AO5" s="19"/>
+      <c r="AP5" s="19"/>
+      <c r="AQ5" s="19"/>
+      <c r="AR5" s="19"/>
+      <c r="AS5" s="19"/>
+      <c r="AT5" s="19"/>
+      <c r="AU5" s="19"/>
+      <c r="AV5" s="19"/>
+      <c r="AW5" s="19"/>
       <c r="AX5" s="2">
         <v>1</v>
       </c>
@@ -1534,13 +1544,13 @@
       </c>
     </row>
     <row r="6" spans="2:79" ht="35.25" x14ac:dyDescent="0.7">
-      <c r="B6" s="13"/>
-      <c r="C6" s="13"/>
-      <c r="D6" s="13"/>
-      <c r="E6" s="13"/>
-      <c r="F6" s="13"/>
-      <c r="G6" s="13"/>
-      <c r="H6" s="13"/>
+      <c r="B6" s="19"/>
+      <c r="C6" s="19"/>
+      <c r="D6" s="19"/>
+      <c r="E6" s="19"/>
+      <c r="F6" s="19"/>
+      <c r="G6" s="19"/>
+      <c r="H6" s="19"/>
       <c r="I6" s="3" t="s">
         <v>77</v>
       </c>
@@ -1622,8 +1632,8 @@
       <c r="AI6" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="AJ6" s="13"/>
-      <c r="AK6" s="13"/>
+      <c r="AJ6" s="19"/>
+      <c r="AK6" s="19"/>
       <c r="AL6" s="1" t="s">
         <v>39</v>
       </c>
@@ -1859,7 +1869,7 @@
         <v>46044</v>
       </c>
       <c r="AK7" s="8" t="str">
-        <f>AK12</f>
+        <f>AK10</f>
         <v>条件式
 結果</v>
       </c>
@@ -2060,7 +2070,7 @@
     </row>
     <row r="9" spans="2:79" x14ac:dyDescent="0.7">
       <c r="B9" s="6">
-        <f t="shared" ref="B9:C11" si="2">B7</f>
+        <f t="shared" ref="B9:C9" si="2">B7</f>
         <v>24</v>
       </c>
       <c r="C9" s="6">
@@ -2068,7 +2078,7 @@
         <v>1019</v>
       </c>
       <c r="D9" s="6">
-        <f t="shared" ref="D9:H11" si="3">D7</f>
+        <f t="shared" ref="D9:H9" si="3">D7</f>
         <v>1</v>
       </c>
       <c r="E9" s="6" t="str">
@@ -2095,7 +2105,7 @@
         <v>46023</v>
       </c>
       <c r="K9" s="9">
-        <f t="shared" ref="K9:O11" si="4">K7</f>
+        <f t="shared" ref="K9:O9" si="4">K7</f>
         <v>46024</v>
       </c>
       <c r="L9" s="9" t="str">
@@ -2190,91 +2200,80 @@
       <c r="BZ9" s="2"/>
       <c r="CA9" s="2"/>
     </row>
-    <row r="10" spans="2:79" x14ac:dyDescent="0.7">
-      <c r="B10" s="6">
-        <f t="shared" si="2"/>
-        <v>24</v>
-      </c>
-      <c r="C10" s="6">
-        <f t="shared" si="2"/>
-        <v>1019</v>
-      </c>
-      <c r="D10" s="6">
-        <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="E10" s="6" t="str">
-        <f t="shared" si="3"/>
-        <v>Aさん</v>
-      </c>
-      <c r="F10" s="6" t="str">
-        <f t="shared" si="3"/>
-        <v>Bさん</v>
-      </c>
-      <c r="G10" s="6" t="str">
-        <f t="shared" si="3"/>
-        <v>Cさん</v>
-      </c>
-      <c r="H10" s="6" t="str">
-        <f t="shared" si="3"/>
-        <v>Dさん</v>
-      </c>
+    <row r="10" spans="2:79" ht="52.9" x14ac:dyDescent="0.7">
+      <c r="B10" s="6"/>
+      <c r="C10" s="6"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="6"/>
+      <c r="G10" s="6"/>
+      <c r="H10" s="6"/>
       <c r="I10" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="J10" s="9">
-        <f>J8</f>
-        <v>46023</v>
-      </c>
-      <c r="K10" s="9">
-        <f t="shared" si="4"/>
-        <v>46024</v>
-      </c>
-      <c r="L10" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v>プルダウン
-決定／概算</v>
-      </c>
-      <c r="M10" s="9">
-        <f t="shared" si="4"/>
-        <v>46025</v>
-      </c>
-      <c r="N10" s="9">
-        <f t="shared" si="4"/>
-        <v>46026</v>
-      </c>
-      <c r="O10" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v>プルダウン
-暫定／調整中／済み</v>
-      </c>
-      <c r="P10" s="5"/>
-      <c r="Q10" s="5"/>
-      <c r="R10" s="6"/>
-      <c r="S10" s="6"/>
-      <c r="T10" s="5"/>
-      <c r="U10" s="5"/>
-      <c r="V10" s="5"/>
-      <c r="W10" s="5"/>
-      <c r="X10" s="5"/>
-      <c r="Y10" s="5"/>
-      <c r="Z10" s="5"/>
-      <c r="AA10" s="5"/>
-      <c r="AB10" s="5"/>
-      <c r="AC10" s="5"/>
-      <c r="AD10" s="5"/>
-      <c r="AE10" s="5"/>
-      <c r="AF10" s="5"/>
+        <v>80</v>
+      </c>
+      <c r="J10" s="9"/>
+      <c r="K10" s="6"/>
+      <c r="L10" s="6"/>
+      <c r="M10" s="6"/>
+      <c r="N10" s="6"/>
+      <c r="O10" s="6"/>
+      <c r="P10" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="Q10" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="R10" s="12"/>
+      <c r="S10" s="12"/>
+      <c r="T10" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="U10" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="V10" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="W10" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="X10" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="Y10" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="Z10" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="AA10" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="AB10" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="AC10" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="AD10" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="AE10" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="AF10" s="11" t="s">
+        <v>78</v>
+      </c>
       <c r="AG10" s="6"/>
       <c r="AH10" s="11" t="s">
-        <v>82</v>
-      </c>
-      <c r="AI10" s="5"/>
+        <v>78</v>
+      </c>
+      <c r="AI10" s="11" t="s">
+        <v>78</v>
+      </c>
       <c r="AJ10" s="6"/>
-      <c r="AK10" s="6" t="str">
-        <f t="shared" ref="AK10:AK11" si="5">AK9</f>
-        <v>条件式
-結果</v>
+      <c r="AK10" s="11" t="s">
+        <v>79</v>
       </c>
       <c r="AL10" s="6"/>
       <c r="AM10" s="6"/>
@@ -2287,7 +2286,10 @@
       <c r="AT10" s="10"/>
       <c r="AU10" s="10"/>
       <c r="AV10" s="10"/>
-      <c r="AW10" s="6"/>
+      <c r="AW10" s="6" t="str">
+        <f>IF(ISBLANK(AW7),"",AW7)</f>
+        <v/>
+      </c>
       <c r="AX10" s="2"/>
       <c r="AY10" s="2"/>
       <c r="AZ10" s="2"/>
@@ -2320,269 +2322,37 @@
       <c r="CA10" s="2"/>
     </row>
     <row r="11" spans="2:79" x14ac:dyDescent="0.7">
-      <c r="B11" s="6">
-        <f t="shared" si="2"/>
-        <v>24</v>
-      </c>
-      <c r="C11" s="6">
-        <f t="shared" si="2"/>
-        <v>1019</v>
-      </c>
-      <c r="D11" s="6">
-        <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="E11" s="6" t="str">
-        <f t="shared" si="3"/>
-        <v>Aさん</v>
-      </c>
-      <c r="F11" s="6" t="str">
-        <f t="shared" si="3"/>
-        <v>Bさん</v>
-      </c>
-      <c r="G11" s="6" t="str">
-        <f t="shared" si="3"/>
-        <v>Cさん</v>
-      </c>
-      <c r="H11" s="6" t="str">
-        <f t="shared" si="3"/>
-        <v>Dさん</v>
-      </c>
-      <c r="I11" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="J11" s="9">
-        <f>J9</f>
-        <v>46023</v>
-      </c>
-      <c r="K11" s="9">
-        <f t="shared" si="4"/>
-        <v>46024</v>
-      </c>
-      <c r="L11" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v>プルダウン
-決定／概算</v>
-      </c>
-      <c r="M11" s="9">
-        <f t="shared" si="4"/>
-        <v>46025</v>
-      </c>
-      <c r="N11" s="9">
-        <f t="shared" si="4"/>
-        <v>46026</v>
-      </c>
-      <c r="O11" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v>プルダウン
-暫定／調整中／済み</v>
-      </c>
-      <c r="P11" s="5"/>
-      <c r="Q11" s="5"/>
-      <c r="R11" s="6"/>
-      <c r="S11" s="6"/>
-      <c r="T11" s="5"/>
-      <c r="U11" s="5"/>
-      <c r="V11" s="5"/>
-      <c r="W11" s="5"/>
-      <c r="X11" s="5"/>
-      <c r="Y11" s="5"/>
-      <c r="Z11" s="5"/>
-      <c r="AA11" s="5"/>
-      <c r="AB11" s="5"/>
-      <c r="AC11" s="5"/>
-      <c r="AD11" s="5"/>
-      <c r="AE11" s="5"/>
-      <c r="AF11" s="5"/>
-      <c r="AG11" s="6"/>
-      <c r="AH11" s="11" t="s">
-        <v>82</v>
-      </c>
-      <c r="AI11" s="5"/>
-      <c r="AJ11" s="6"/>
-      <c r="AK11" s="6" t="str">
-        <f t="shared" si="5"/>
-        <v>条件式
-結果</v>
-      </c>
-      <c r="AL11" s="6"/>
-      <c r="AM11" s="6"/>
-      <c r="AN11" s="6"/>
-      <c r="AO11" s="6"/>
-      <c r="AP11" s="10"/>
-      <c r="AQ11" s="10"/>
-      <c r="AR11" s="10"/>
-      <c r="AS11" s="10"/>
-      <c r="AT11" s="10"/>
-      <c r="AU11" s="10"/>
-      <c r="AV11" s="10"/>
-      <c r="AW11" s="6"/>
-      <c r="AX11" s="2"/>
-      <c r="AY11" s="2"/>
-      <c r="AZ11" s="2"/>
-      <c r="BA11" s="2"/>
-      <c r="BB11" s="2"/>
-      <c r="BC11" s="2"/>
-      <c r="BD11" s="2"/>
-      <c r="BE11" s="2"/>
-      <c r="BF11" s="2"/>
-      <c r="BG11" s="2"/>
-      <c r="BH11" s="2"/>
-      <c r="BI11" s="2"/>
-      <c r="BJ11" s="2"/>
-      <c r="BK11" s="2"/>
-      <c r="BL11" s="2"/>
-      <c r="BM11" s="2"/>
-      <c r="BN11" s="2"/>
-      <c r="BO11" s="2"/>
-      <c r="BP11" s="2"/>
-      <c r="BQ11" s="2"/>
-      <c r="BR11" s="2"/>
-      <c r="BS11" s="2"/>
-      <c r="BT11" s="2"/>
-      <c r="BU11" s="2"/>
-      <c r="BV11" s="2"/>
-      <c r="BW11" s="2"/>
-      <c r="BX11" s="2"/>
-      <c r="BY11" s="2"/>
-      <c r="BZ11" s="2"/>
-      <c r="CA11" s="2"/>
+      <c r="J11" s="4"/>
     </row>
-    <row r="12" spans="2:79" ht="52.9" x14ac:dyDescent="0.7">
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="J12" s="9"/>
-      <c r="K12" s="6"/>
-      <c r="L12" s="6"/>
-      <c r="M12" s="6"/>
-      <c r="N12" s="6"/>
-      <c r="O12" s="6"/>
-      <c r="P12" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="Q12" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="R12" s="12"/>
-      <c r="S12" s="12"/>
-      <c r="T12" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="U12" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="V12" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="W12" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="X12" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="Y12" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="Z12" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="AA12" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="AB12" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="AC12" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="AD12" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="AE12" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="AF12" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="AG12" s="6"/>
-      <c r="AH12" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="AI12" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="AJ12" s="6"/>
-      <c r="AK12" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="AL12" s="6"/>
-      <c r="AM12" s="6"/>
-      <c r="AN12" s="6"/>
-      <c r="AO12" s="6"/>
-      <c r="AP12" s="10"/>
-      <c r="AQ12" s="10"/>
-      <c r="AR12" s="10"/>
-      <c r="AS12" s="10"/>
-      <c r="AT12" s="10"/>
-      <c r="AU12" s="10"/>
-      <c r="AV12" s="10"/>
-      <c r="AW12" s="6" t="str">
-        <f>IF(ISBLANK(AW7),"",AW7)</f>
-        <v/>
-      </c>
-      <c r="AX12" s="2"/>
-      <c r="AY12" s="2"/>
-      <c r="AZ12" s="2"/>
-      <c r="BA12" s="2"/>
-      <c r="BB12" s="2"/>
-      <c r="BC12" s="2"/>
-      <c r="BD12" s="2"/>
-      <c r="BE12" s="2"/>
-      <c r="BF12" s="2"/>
-      <c r="BG12" s="2"/>
-      <c r="BH12" s="2"/>
-      <c r="BI12" s="2"/>
-      <c r="BJ12" s="2"/>
-      <c r="BK12" s="2"/>
-      <c r="BL12" s="2"/>
-      <c r="BM12" s="2"/>
-      <c r="BN12" s="2"/>
-      <c r="BO12" s="2"/>
-      <c r="BP12" s="2"/>
-      <c r="BQ12" s="2"/>
-      <c r="BR12" s="2"/>
-      <c r="BS12" s="2"/>
-      <c r="BT12" s="2"/>
-      <c r="BU12" s="2"/>
-      <c r="BV12" s="2"/>
-      <c r="BW12" s="2"/>
-      <c r="BX12" s="2"/>
-      <c r="BY12" s="2"/>
-      <c r="BZ12" s="2"/>
-      <c r="CA12" s="2"/>
+    <row r="12" spans="2:79" x14ac:dyDescent="0.7">
+      <c r="J12" s="4"/>
     </row>
     <row r="13" spans="2:79" x14ac:dyDescent="0.7">
       <c r="J13" s="4"/>
     </row>
     <row r="14" spans="2:79" x14ac:dyDescent="0.7">
+      <c r="H14" t="s">
+        <v>87</v>
+      </c>
       <c r="J14" s="4"/>
     </row>
     <row r="15" spans="2:79" x14ac:dyDescent="0.7">
-      <c r="J15" s="4"/>
+      <c r="H15" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="16" spans="2:79" x14ac:dyDescent="0.7">
-      <c r="J16" s="4"/>
+      <c r="H16" t="s">
+        <v>89</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="AX4:CA4"/>
+    <mergeCell ref="AE5:AG5"/>
+    <mergeCell ref="AJ5:AJ6"/>
+    <mergeCell ref="AK5:AK6"/>
+    <mergeCell ref="AX3:CA3"/>
     <mergeCell ref="B3:H4"/>
     <mergeCell ref="I3:AK4"/>
     <mergeCell ref="AL3:AW5"/>
@@ -2596,11 +2366,6 @@
     <mergeCell ref="E5:E6"/>
     <mergeCell ref="F5:F6"/>
     <mergeCell ref="G5:G6"/>
-    <mergeCell ref="AX4:CA4"/>
-    <mergeCell ref="AE5:AG5"/>
-    <mergeCell ref="AJ5:AJ6"/>
-    <mergeCell ref="AK5:AK6"/>
-    <mergeCell ref="AX3:CA3"/>
   </mergeCells>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>